<commit_message>
docs(events): v1.4 shipped three states, not one
Andi confirms two unofficial releases after the v1.4.1 tag. Git records them
unevenly: 1.4.2 is visible (@version 1.4.2 in aGTM.js from 598776d 2025-09-09
through 081b3df, plus the sGTM client template and a CHANGELOG entry, never
tagged, never on main), while 1.4.3pre appears nowhere as a version — no commit
carries it, the name only exists in prose.

For the event reference this barely matters, and saying so is the point: the
form/scroll/click templates are byte-identical across the whole v1.4 line, and
the three breaking changes came with the tag hardening in July 2026, i.e. after
all of it. What does differ is the two variable templates, which arrived with
1.4.2 — the doc no longer claims they ship with v1.5.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/aGTM-Events-v1.4.xlsx
+++ b/assets/aGTM-Events-v1.4.xlsx
@@ -4399,7 +4399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4529,82 +4529,94 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Only one variable template</t>
+          <t>Which v1.4 exactly</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>v1.4.1 ships only aGTM var - Content Counter. The Consent-Check and Consent-Info variables were added afterwards (CHANGELOG entry 1.4.2, never tagged/released) and ship with v1.5.</t>
+          <t>This sheet describes v1.4.1, the last TAGGED release. Two later states shipped unofficially without a tag: 1.4.2 (aGTM.js carries @version 1.4.2 from 2025-09-09 until the v1.5 bump) and 1.4.3pre, which git does not record as a version at all. The events and attributes below apply to all three - they differ in CMP adapters, variable templates and build tooling, not in events.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>No per-event flags</t>
+          <t>Variable templates differ</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>The flags _noConsent, _noDLPush and _post (POST transport) are v1.5 only. In v1.4.x every non-aGTM* event is consent-gated, without exception.</t>
+          <t>v1.4.1 ships only aGTM var - Content Counter; aGTM var - Consent Check and aGTM var - Consent Info came with the unofficial 1.4.2. Whether you have them depends on which of the three states you run.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>aGTM_consent_update is not gated</t>
+          <t>No per-event flags</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>In v1.4.x the event fires on every run_cc('update') run. v1.5 only fires it on a changed consent state (hash gating).</t>
+          <t>The flags _noConsent, _noDLPush and _post (POST transport) are v1.5 only. In v1.4.x every non-aGTM* event is consent-gated, without exception.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>No session/attribution/bot data</t>
+          <t>aGTM_consent_update is not gated</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>aGTM.d.session, aGTM.d.attribution and aGTM.d.bot come with the v1.5 sGTM Client. In v1.4.x only aGTM.d.consent, aGTM.d.dl and aGTM.l exist.</t>
+          <t>In v1.4.x the event fires on every run_cc('update') run. v1.5 only fires it on a changed consent state (hash gating).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
+          <t>No session/attribution/bot data</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>aGTM.d.session, aGTM.d.attribution and aGTM.d.bot come with the v1.5 sGTM Client. In v1.4.x only aGTM.d.consent, aGTM.d.dl and aGTM.l exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
           <t>DL-Repeat is tag-only</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>The replay engine (gate wait, poll, late enrichment, aGTM_repeat_fallback) moved into the library with v1.5. The v1.4.x tag only marks replayed events with aGTMrepeated = true.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>aGTM version</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>v1.4  (DEPRECATED)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
+          <t>aGTM version</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>v1.4  (DEPRECATED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Generated from the aGTM sources (aGTM.js + gtm/**/*.tpl). Companion to EVENTS-v1.4.md in the repository, which additionally covers the consent gate, the event flags and the aGTM.* JavaScript paths.</t>
         </is>

</xml_diff>